<commit_message>
Updated nutrition and modules by programme
</commit_message>
<xml_diff>
--- a/Modules by programme.xlsx
+++ b/Modules by programme.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ljmu.sharepoint.com/teams/SPSRe-validation2026Team/Shared Documents/General/Core Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="85" documentId="8_{8B61065D-E51E-403C-80DC-4765F6BBB67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1ADC4786-F63B-DD4B-8B29-A7C5B5C46610}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{8B61065D-E51E-403C-80DC-4765F6BBB67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F31DA471-4A88-4276-8861-1E62C2BEFC7A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{2784CFB3-2F37-4B03-A558-B52980BC9FFA}"/>
+    <workbookView xWindow="14775" yWindow="0" windowWidth="14130" windowHeight="15585" xr2:uid="{2784CFB3-2F37-4B03-A558-B52980BC9FFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="172">
   <si>
     <t>S&amp;F</t>
   </si>
@@ -83,7 +83,7 @@
     <t>Learning Theory and Practice 1</t>
   </si>
   <si>
-    <t>4NX1SPS</t>
+    <t>4001SPS</t>
   </si>
   <si>
     <t>Professional Practice 1 in Sport Nutrition</t>
@@ -113,7 +113,7 @@
     <t xml:space="preserve">Professional Practice in Sport Coaching 1 </t>
   </si>
   <si>
-    <t>4NX2SPS</t>
+    <t>4003SPS</t>
   </si>
   <si>
     <t>Principles of Human Nutrition</t>
@@ -149,7 +149,7 @@
     <t>Professional Practice in Sport Coaching 2</t>
   </si>
   <si>
-    <t>4NX3SPS</t>
+    <t>4004SPS</t>
   </si>
   <si>
     <t>Nutritional Biochemistry and Metabolism</t>
@@ -167,91 +167,97 @@
     <t>Football tactics and match analysis</t>
   </si>
   <si>
+    <t>5203SPS</t>
+  </si>
+  <si>
+    <t>Primary PE teacher Education</t>
+  </si>
+  <si>
+    <t>4092SPS</t>
+  </si>
+  <si>
+    <t>Exercise Phys L4</t>
+  </si>
+  <si>
+    <t>5402SPS</t>
+  </si>
+  <si>
+    <t>Effective Coaching in Paralympic and Disability Sport</t>
+  </si>
+  <si>
+    <t>4006SPS</t>
+  </si>
+  <si>
+    <t>Performance Nutrition</t>
+  </si>
+  <si>
+    <t>4054SPS</t>
+  </si>
+  <si>
+    <t>Academic Skills</t>
+  </si>
+  <si>
+    <t>6301SPS</t>
+  </si>
+  <si>
+    <t>Football Performance and Technology</t>
+  </si>
+  <si>
+    <t>5204SPS</t>
+  </si>
+  <si>
+    <t>Physical Education in Action 1</t>
+  </si>
+  <si>
+    <t>4094SPS</t>
+  </si>
+  <si>
+    <t>Human Movement</t>
+  </si>
+  <si>
+    <t>5403SPS</t>
+  </si>
+  <si>
+    <t>Strength and Conditioning for Coaches</t>
+  </si>
+  <si>
+    <t>5001SPS</t>
+  </si>
+  <si>
+    <t>Professional Practice 2 in Sport Nutrition</t>
+  </si>
+  <si>
+    <t>4093SPS</t>
+  </si>
+  <si>
+    <t>Psychosocial Principles of Sport and Exercise</t>
+  </si>
+  <si>
+    <t>6302SPS</t>
+  </si>
+  <si>
+    <t>Physical Performance in Football</t>
+  </si>
+  <si>
+    <t>6201SPS</t>
+  </si>
+  <si>
+    <t>PE in Action 2</t>
+  </si>
+  <si>
+    <t>5091SPS</t>
+  </si>
+  <si>
+    <t>Research Methods 2</t>
+  </si>
+  <si>
     <t>5202SPS</t>
   </si>
   <si>
-    <t>4092SPS</t>
-  </si>
-  <si>
-    <t>Exercise Phys L4</t>
-  </si>
-  <si>
-    <t>5402SPS</t>
-  </si>
-  <si>
-    <t>Effective Coaching in Paralympic and Disability Sport</t>
-  </si>
-  <si>
-    <t>4NX4SPS</t>
-  </si>
-  <si>
-    <t>Performance Nutrition</t>
-  </si>
-  <si>
-    <t>4054SPS</t>
-  </si>
-  <si>
-    <t>Academic Skills</t>
-  </si>
-  <si>
-    <t>6301SPS</t>
-  </si>
-  <si>
-    <t>Football Performance and Technology</t>
-  </si>
-  <si>
-    <t>5203SPS</t>
-  </si>
-  <si>
-    <t>Primary PE teacher Education</t>
-  </si>
-  <si>
-    <t>4094SPS</t>
-  </si>
-  <si>
-    <t>Human Movement</t>
-  </si>
-  <si>
-    <t>5403SPS</t>
-  </si>
-  <si>
-    <t>Strength and Conditioning for Coaches</t>
-  </si>
-  <si>
-    <t>5NX1SPS</t>
-  </si>
-  <si>
-    <t>Professional Practice 2 in Sport Nutrition</t>
-  </si>
-  <si>
-    <t>4093SPS</t>
-  </si>
-  <si>
-    <t>Psychosocial Principles of Sport and Exercise</t>
-  </si>
-  <si>
-    <t>6302SPS</t>
-  </si>
-  <si>
-    <t>Physical Performance in Football</t>
-  </si>
-  <si>
-    <t>5204SPS</t>
-  </si>
-  <si>
-    <t>Physical Education in Action 1</t>
-  </si>
-  <si>
-    <t>5091SPS</t>
-  </si>
-  <si>
-    <t>Research Methods 2</t>
-  </si>
-  <si>
-    <t>Learning Theory and Practice</t>
-  </si>
-  <si>
-    <t>5NX2SPS</t>
+    <t>Learning Theory and Practice 2</t>
+  </si>
+  <si>
+    <t>5014SPS</t>
   </si>
   <si>
     <t>Product Development for Sport Nutrition</t>
@@ -272,19 +278,25 @@
     <t>6202SPS</t>
   </si>
   <si>
+    <t>Learning Theory and Practice 3</t>
+  </si>
+  <si>
     <t>5092SPS</t>
   </si>
   <si>
     <t>Physiological adaptations to exercise</t>
   </si>
   <si>
+    <t>5405SPS</t>
+  </si>
+  <si>
     <t>Youth and Community Football Coaching</t>
   </si>
   <si>
-    <t>5NX3SPS</t>
-  </si>
-  <si>
-    <t>Applied Nutrition and Exercise Biochemistry</t>
+    <t>5015SPS</t>
+  </si>
+  <si>
+    <t>Exercise Biochemistry</t>
   </si>
   <si>
     <t>5052SPS</t>
@@ -311,52 +323,82 @@
     <t>Professional Practice in Sport and Exercise Science 2</t>
   </si>
   <si>
+    <t>5094SPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sport PE and society </t>
+  </si>
+  <si>
+    <t>5005SPS</t>
+  </si>
+  <si>
+    <t>Lifespan Nutrition and Eating Behaviour</t>
+  </si>
+  <si>
+    <t>5053SPS</t>
+  </si>
+  <si>
+    <t>Exercise and Health Psychology</t>
+  </si>
+  <si>
+    <t>6096SPS</t>
+  </si>
+  <si>
+    <t>Secondary PE Teacher Education</t>
+  </si>
+  <si>
+    <t>5102SPS</t>
+  </si>
+  <si>
+    <t>Influences and Assessment of Physical Activity and Sedentary Behaviour</t>
+  </si>
+  <si>
+    <t>6401SPS</t>
+  </si>
+  <si>
     <t xml:space="preserve">Advanced Coaching Practice </t>
   </si>
   <si>
-    <t>5NX4SPS</t>
-  </si>
-  <si>
-    <t>Lifespan Nutrition and Eating Behaviour</t>
-  </si>
-  <si>
-    <t>5053SPS</t>
-  </si>
-  <si>
-    <t>Exercise and Health Psychology</t>
-  </si>
-  <si>
-    <t>6096SPS</t>
-  </si>
-  <si>
-    <t>Secondary PE Teacher Education</t>
-  </si>
-  <si>
-    <t>5102SPS</t>
-  </si>
-  <si>
-    <t>Influences and Assessment of Physical Activity and Sedentary Behaviour</t>
+    <t>6003SPS</t>
+  </si>
+  <si>
+    <t>Molecular Nutrition and Genetics</t>
+  </si>
+  <si>
+    <t>5054SPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developmental and Social Psychology </t>
+  </si>
+  <si>
+    <t>5103SPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biomechanics </t>
+  </si>
+  <si>
+    <t>6402SPS</t>
   </si>
   <si>
     <t xml:space="preserve">Coach Development and Learning </t>
   </si>
   <si>
-    <t>6NX1SPS</t>
-  </si>
-  <si>
-    <t>Molecular Nutrition and Genetics</t>
-  </si>
-  <si>
-    <t>5054SPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developmental and Social Psychology </t>
-  </si>
-  <si>
-    <t>5103SPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biomechanics </t>
+    <t>6004SPS</t>
+  </si>
+  <si>
+    <t>Sport Supplements and Contemporary Issues</t>
+  </si>
+  <si>
+    <t>5093SPS</t>
+  </si>
+  <si>
+    <t>Sport and Performance Psychology</t>
+  </si>
+  <si>
+    <t>6101SPS</t>
+  </si>
+  <si>
+    <t>Sport and Injury Biomechanics</t>
   </si>
   <si>
     <t>6403SPS</t>
@@ -365,22 +407,22 @@
     <t xml:space="preserve">Placement/Projects in Sport for Professional Development </t>
   </si>
   <si>
-    <t>6NX2SPS</t>
-  </si>
-  <si>
-    <t>Sport Supplements and Contemporary Issues</t>
-  </si>
-  <si>
-    <t>5093SPS</t>
-  </si>
-  <si>
-    <t>Sport and Performance Psychology</t>
-  </si>
-  <si>
-    <t>6101SPS</t>
-  </si>
-  <si>
-    <t>Sport and Injury Biomechanics</t>
+    <t>6007SPS</t>
+  </si>
+  <si>
+    <t>Sport Nutrition for Health, Adaptation and Recovery</t>
+  </si>
+  <si>
+    <t>6051SPS</t>
+  </si>
+  <si>
+    <t>Professional Practice 3</t>
+  </si>
+  <si>
+    <t>6102SPS</t>
+  </si>
+  <si>
+    <t>Physical activity and sedentary behaviour across the life course</t>
   </si>
   <si>
     <t>6097SPS</t>
@@ -389,25 +431,7 @@
     <t>Working in High Performance Sport</t>
   </si>
   <si>
-    <t>6NX3SPS</t>
-  </si>
-  <si>
-    <t>Sport Nutrition for Health, Adaptation and Recovery</t>
-  </si>
-  <si>
-    <t>6051SPS</t>
-  </si>
-  <si>
-    <t>Professional Practice 3</t>
-  </si>
-  <si>
-    <t>6102SPS</t>
-  </si>
-  <si>
-    <t>Physical activity and sedentary behaviour across the life course</t>
-  </si>
-  <si>
-    <t>6NX4SPS</t>
+    <t>6008SPS</t>
   </si>
   <si>
     <t xml:space="preserve">Capstone Placment Project </t>
@@ -425,10 +449,10 @@
     <t>Exercise Metabolism</t>
   </si>
   <si>
-    <t>6NX5SPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applied Placement </t>
+    <t>6006SPS</t>
+  </si>
+  <si>
+    <t>Applied Placement  (currently 6006SPS)</t>
   </si>
   <si>
     <t>6053SPS</t>
@@ -503,6 +527,18 @@
     <t>Performance Analysis in Sport</t>
   </si>
   <si>
+    <t>Study Abroad</t>
+  </si>
+  <si>
+    <t>Year / Semester</t>
+  </si>
+  <si>
+    <t>Aim for one across all progs</t>
+  </si>
+  <si>
+    <t>Sandwich Year</t>
+  </si>
+  <si>
     <t xml:space="preserve"> "https://ljmu.sharepoint.com/teams/SPSRe-validation2026Team/Shared Documents/Football Science/Module Documents"</t>
   </si>
   <si>
@@ -519,43 +555,13 @@
   </si>
   <si>
     <t xml:space="preserve"> "https://ljmu.sharepoint.com/teams/SPSRe-validation2026Team/Shared Documents/Sport Psychology/Module Documents"</t>
-  </si>
-  <si>
-    <t>5404SPS</t>
-  </si>
-  <si>
-    <t>5405SPS</t>
-  </si>
-  <si>
-    <t>6405SPS</t>
-  </si>
-  <si>
-    <t>6404SPS</t>
-  </si>
-  <si>
-    <t>Applied Placement in Football Science</t>
-  </si>
-  <si>
-    <t>Learning Theory and Practice 2</t>
-  </si>
-  <si>
-    <t>Sport PE and Society</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sport PE and society </t>
-  </si>
-  <si>
-    <t>Learning Theory and Practice 3</t>
-  </si>
-  <si>
-    <t>PE in Action 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -626,6 +632,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -653,7 +675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -666,12 +688,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1008,9 +1029,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F437026B-C1B6-43E1-9BC1-A61C107F7F08}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B4:AI40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <sheetData>
-    <row r="4" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:35">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1030,7 +1051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:35">
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
@@ -1055,7 +1076,7 @@
       <c r="V5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AB5" s="10" t="s">
+      <c r="AB5" s="6" t="s">
         <v>14</v>
       </c>
       <c r="AC5" s="6" t="s">
@@ -1068,7 +1089,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:35">
       <c r="B6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1093,7 +1114,7 @@
       <c r="V6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="AB6" s="10" t="s">
+      <c r="AB6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="AC6" s="6" t="s">
@@ -1106,7 +1127,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:35">
       <c r="B7" s="4" t="s">
         <v>28</v>
       </c>
@@ -1131,7 +1152,7 @@
       <c r="V7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AB7" s="6" t="s">
         <v>36</v>
       </c>
       <c r="AC7" s="6" t="s">
@@ -1144,7 +1165,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:35">
       <c r="B8" s="4" t="s">
         <v>40</v>
       </c>
@@ -1155,404 +1176,401 @@
         <v>42</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>165</v>
+        <v>43</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="V8" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB8" s="10" t="s">
         <v>47</v>
       </c>
+      <c r="AB8" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="AC8" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AH8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AI8" s="7" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="2:35" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="2:35">
       <c r="B9" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V9" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB9" s="10" t="s">
         <v>59</v>
       </c>
+      <c r="AB9" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="AC9" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AH9" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AI9" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="2:35" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="2:35">
       <c r="B10" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="U10" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="V10" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="AB10" s="10" t="s">
+      <c r="U10" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="V10" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB10" s="11" t="s">
+        <v>72</v>
+      </c>
       <c r="AC10" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="AH10" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AI10" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="2:35" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="2:35">
       <c r="B11" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>168</v>
+        <v>79</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="U11" s="9" t="s">
-        <v>161</v>
+        <v>81</v>
+      </c>
+      <c r="U11" s="12" t="s">
+        <v>82</v>
       </c>
       <c r="V11" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="AB11" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
+      </c>
+      <c r="AB11" s="11" t="s">
+        <v>84</v>
       </c>
       <c r="AC11" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="AH11" s="7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="AI11" s="7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="2:35" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="2:35">
       <c r="B12" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="U12" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="V12" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB12" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
+      </c>
+      <c r="U12" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="V12" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="AB12" s="6" t="s">
+        <v>96</v>
       </c>
       <c r="AC12" s="6" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AH12" s="7" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="AI12" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="2:35" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="2:35">
       <c r="H13" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="U13" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="V13" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="AB13" s="10" t="s">
-        <v>100</v>
+        <v>103</v>
+      </c>
+      <c r="U13" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="V13" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB13" s="6" t="s">
+        <v>106</v>
       </c>
       <c r="AC13" s="6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="AH13" s="7" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="AI13" s="7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" spans="2:35" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="2:35">
       <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I14" s="15" t="s">
-        <v>169</v>
-      </c>
       <c r="N14" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="V14" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="AB14" s="10" t="s">
-        <v>108</v>
+        <v>113</v>
+      </c>
+      <c r="AB14" s="6" t="s">
+        <v>114</v>
       </c>
       <c r="AC14" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="AH14" s="7" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="AI14" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="2:35" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="2:35">
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="U15" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="V15" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="AB15" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH15" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="AI15" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="2:35">
+      <c r="B16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="U16" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="V16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB16" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="AC16" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH16" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="AI16" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="2:35">
+      <c r="B17" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N15" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="U15" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="V15" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="AB15" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AC15" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="AH15" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AI15" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="16" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="B16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="I17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="AB17" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="AC17" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="AH17" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AI17" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="2:35">
+      <c r="H18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I16" s="7" t="s">
+      <c r="I18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="U18" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="N16" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB16" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC16" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="AH16" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="AI16" s="7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="17" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="B17" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H17" s="2" t="s">
+      <c r="V18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AH18" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="AI18" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="2:35">
+      <c r="B19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="U19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="V19" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="U17" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="V17" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB17" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="AC17" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="AH17" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="AI17" s="7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="18" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="U18" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="V18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AH18" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="AI18" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="B19" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="U19" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="V19" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="AB19" s="2" t="s">
         <v>32</v>
@@ -1561,30 +1579,36 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:35">
       <c r="B20" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="O20" s="11" t="s">
-        <v>139</v>
+        <v>146</v>
+      </c>
+      <c r="O20" s="10" t="s">
+        <v>147</v>
       </c>
       <c r="U20" s="2" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="AB20" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AC20" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH20" s="2" t="s">
         <v>32</v>
@@ -1593,236 +1617,269 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="2:35" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:35">
       <c r="B21" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="I21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="U21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AH21" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="N21" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="O21" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="AB21" s="2"/>
-      <c r="AC21" s="2"/>
-      <c r="AH21" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="AI21" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="2:35">
+      <c r="B22" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="AB22" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC22" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="2:35">
+      <c r="H23" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="AB23" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="B22" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="U22" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="V22" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H23" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="V23" t="s">
+      <c r="AC23" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" spans="2:35">
+      <c r="B24" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="2:35">
+      <c r="B25" s="13"/>
+      <c r="C25" s="14"/>
+      <c r="N25" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB25" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="AC25" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="AH25" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="AI25" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="26" spans="2:35">
+      <c r="H26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O26" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="U26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="V26" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" spans="2:35">
+      <c r="H27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="U27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="V27" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="2:35">
+      <c r="H28" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="2:35">
+      <c r="H29" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N29" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="O29" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="2:35">
+      <c r="H30" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="N30" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="O30" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="31" spans="2:35">
+      <c r="N31" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="O31" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="33" spans="2:34">
+      <c r="N33" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="O33" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="35" spans="2:34">
+      <c r="N35" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="37" spans="2:34">
+      <c r="O37" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="S37" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="38" spans="2:34">
+      <c r="O38" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="S38" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" spans="2:34">
+      <c r="B40" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H40" s="8" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="24" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="B24" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="I24" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="C25" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="U25" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="V25" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="AB25" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AC25" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="AH25" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="AI25" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="26" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H26" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="U26" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="V26" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="27" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H27" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="28" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H28" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="29" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H29" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="N29" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="O29" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="H30" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="N30" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="O30" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="31" spans="2:35" x14ac:dyDescent="0.2">
-      <c r="I31" s="14"/>
-      <c r="N31" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="O31" s="7" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="34" spans="2:34" x14ac:dyDescent="0.2">
-      <c r="N34" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="O34" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="36" spans="2:34" x14ac:dyDescent="0.2">
-      <c r="N36" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="O36" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="2:34" ht="16" x14ac:dyDescent="0.2">
-      <c r="B40" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>155</v>
-      </c>
       <c r="N40" s="8" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="U40" s="8" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="AB40" s="8" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="AH40" s="8" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -1831,6 +1888,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f1436123-e04c-43f8-b7d8-6e3401685a6a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e2acc87f-978a-4c56-9887-574fe2c7e53e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AF5424D8F461E94980DF8EC8486B8636" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bcfcf74337161f6441250f8f4cf7d932">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f1436123-e04c-43f8-b7d8-6e3401685a6a" xmlns:ns3="e2acc87f-978a-4c56-9887-574fe2c7e53e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c081e04d381fea11733dd13b3c4e862f" ns2:_="" ns3:_="">
     <xsd:import namespace="f1436123-e04c-43f8-b7d8-6e3401685a6a"/>
@@ -2017,66 +2094,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f1436123-e04c-43f8-b7d8-6e3401685a6a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e2acc87f-978a-4c56-9887-574fe2c7e53e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CF219CC-0542-4EA6-B641-A664F11067B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f1436123-e04c-43f8-b7d8-6e3401685a6a"/>
-    <ds:schemaRef ds:uri="e2acc87f-978a-4c56-9887-574fe2c7e53e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{376CA5CE-04DF-4650-A618-9B8D469883CE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75232F14-CFBB-4F59-8870-57158CE22014}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75232F14-CFBB-4F59-8870-57158CE22014}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{376CA5CE-04DF-4650-A618-9B8D469883CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="f1436123-e04c-43f8-b7d8-6e3401685a6a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="e2acc87f-978a-4c56-9887-574fe2c7e53e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CF219CC-0542-4EA6-B641-A664F11067B3}"/>
 </file>
</xml_diff>